<commit_message>
Added structural_mesh_viewer_node.py Added template_match_node.py Added camera_layout_viewer_node.py Added surface_mesh_generator_node.py Added remap_node.py Added fft_1d_node.py Added ifft_1d_node.py Added signal_generator_node.py Added time_sync_node.py Added calib_node.py Added stereo_sync_node.py Added image_data_simulator_node.py Added some samples for like image data simulator (generated images)
</commit_message>
<xml_diff>
--- a/samples/tracking01/tracking08.xlsx
+++ b/samples/tracking01/tracking08.xlsx
@@ -450,7 +450,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1788969999.9329748</t>
+          <t>1789981486.8089256</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>65</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>104</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -609,16 +609,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>466</v>
+        <v>512</v>
       </c>
       <c r="E3" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>545</v>
+        <v>578</v>
       </c>
       <c r="G3" t="n">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -643,10 +643,10 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1042</v>
+        <v>1092</v>
       </c>
       <c r="E4" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="F4" t="n">
         <v>219</v>
@@ -847,16 +847,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>472</v>
+        <v>516</v>
       </c>
       <c r="E10" t="n">
-        <v>391</v>
+        <v>375</v>
       </c>
       <c r="F10" t="n">
-        <v>531</v>
+        <v>570</v>
       </c>
       <c r="G10" t="n">
-        <v>322</v>
+        <v>370</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>{"interval_seconds": "1.0", "timer_target": "0", "button_count": 58, "timer_count": 0}</t>
+          <t>{"interval_seconds": "1.0", "timer_target": "0", "button_count": 64, "timer_count": 0}</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>{"x": "20:10:210", "y": "0", "z": "20:10:170", "indexing": "ij", "point_size": 2.0, "point_color": "blue", "line_width": 1.0, "line_color": "black", "marker": "o", "line_style": "solid", "show_points": true, "show_lines": true, "show_x_lines": true, "show_y_lines": true, "show_z_lines": true, "preview_enabled": false}</t>
+          <t>{"x": "20:10:210", "y": "0", "z": "20:10:170", "indexing": "ij", "point_size": 2.0, "point_color": "blue", "line_width": 1.0, "line_color": "black", "marker": "o", "line_style": "solid", "show_points": true, "show_lines": true, "show_x_lines": true, "show_y_lines": true, "show_z_lines": true, "preview_enabled": true}</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E28" t="n">
         <v>2064</v>
@@ -1472,7 +1472,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>{"method": "folder", "pattern": "..\\..\\..\\..\\..\\ExpDataSamples\\20260100_TimberConnections\\Ling_papper\\20260106_experiment_picture\\First_group_domestic_component\\left_undistorted\\spc1_left_undistorted_%04d.jpg", "start": "0", "end": "100", "pattern_wait": 1.0, "folder": "..\\..\\..\\..\\..\\ExpDataSamples\\20260100_TimberConnections\\Ling_papper\\20260106_experiment_picture\\First_group_domestic_component\\left_undistorted", "file_list": "", "current_index": 0, "fps": "0.5", "batch_start": "1", "batch_end": "500", "batch_step": "1", "batch_current": "500", "batch_frame_1": "1", "batch_frame_2": "i"}</t>
+          <t>{"method": "folder", "pattern": "..\\..\\..\\..\\..\\ExpDataSamples\\20260100_TimberConnections\\Ling_papper\\20260106_experiment_picture\\First_group_domestic_component\\left_undistorted\\spc1_left_undistorted_%04d.jpg", "start": "0", "end": "100", "pattern_wait": 1.0, "folder": "..\\..\\..\\..\\..\\ExpDataSamples\\20260100_TimberConnections\\Ling_papper\\20260106_experiment_picture\\First_group_domestic_component\\left_undistorted", "file_list": "", "current_index": 0, "fps": "0.5", "batch_start": "1", "batch_end": "10", "batch_step": "1", "batch_current": "4", "batch_frame_1": "1", "batch_frame_2": "i"}</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>{"col_names": "col_0, col_1, col_2, col_3, col_4, col_5, col_6, col_7, col_8, col_9, col_10, col_11, col_12, col_13, col_14, col_15, col_16, col_17, col_18, col_19, col_20, col_21, col_22, col_23, col_24, col_25, col_26, col_27, col_28, col_29, col_30, col_31, col_32, col_33, col_34, col_35, col_36, col_37, col_38, col_39, col_40, col_41, col_42, col_43, col_44, col_45, col_46, col_47, col_48, col_49, col_50, col_51, col_52, col_53, col_54, col_55, col_56, col_57, col_58, col_59, col_60, col_61, col_62, col_63, col_64, col_65, col_66, col_67, col_68, col_69, col_70, col_71, col_72, col_73, col_74, col_75, col_76, col_77, col_78, col_79, col_80, col_81, col_82, col_83, col_84, col_85, col_86, col_87, col_88, col_89, col_90, col_91, col_92, col_93, col_94, col_95, col_96, col_97, col_98, col_99, col_100, col_101, col_102, col_103, col_104, col_105, col_106, col_107, col_108, col_109, col_110, col_111, col_112, col_113, col_114, col_115, col_116, col_117, col_118, col_119, col_120, col_121, col_122, col_123, col_124, col_125, col_126, col_127, col_128, col_129, col_130, col_131, col_132, col_133, col_134, col_135, col_136, col_137, col_138, col_139, col_140, col_141, col_142, col_143, col_144, col_145, col_146, col_147, col_148, col_149, col_150, col_151, col_152, col_153, col_154, col_155, col_156, col_157, col_158, col_159, col_160, col_161, col_162, col_163, col_164, col_165, col_166, col_167, col_168, col_169, col_170, col_171, col_172, col_173, col_174, col_175, col_176, col_177, col_178, col_179, col_180, col_181, col_182, col_183, col_184, col_185, col_186, col_187, col_188, col_189, col_190, col_191, col_192, col_193, col_194, col_195, col_196, col_197, col_198, col_199, col_200, col_201, col_202, col_203, col_204, col_205, col_206, col_207, col_208, col_209, col_210, col_211, col_212, col_213, col_214, col_215, col_216, col_217, col_218, col_219, col_220, col_221, col_222, col_223, col_224, col_225, col_226, col_227, col_228, col_229, col_230, col_231, col_232, col_233, col_234, col_235, col_236, col_237, col_238, col_239, col_240, col_241, col_242, col_243, col_244, col_245, col_246, col_247, col_248, col_249, col_250, col_251, col_252, col_253, col_254, col_255, col_256, col_257, col_258, col_259, col_260, col_261, col_262, col_263, col_264, col_265, col_266, col_267, col_268, col_269, col_270, col_271, col_272, col_273, col_274, col_275, col_276, col_277, col_278, col_279, col_280, col_281, col_282, col_283, col_284, col_285, col_286, col_287, col_288, col_289, col_290, col_291, col_292, col_293, col_294, col_295, col_296, col_297, col_298, col_299, col_300, col_301, col_302, col_303, col_304, col_305, col_306, col_307, col_308, col_309, col_310, col_311, col_312, col_313, col_314, col_315, col_316, col_317, col_318, col_319, col_320, col_321, col_322, col_323, col_324, col_325, col_326, col_327, col_328, col_329, col_330, col_331, col_332, col_333, col_334, col_335, col_336, col_337, col_338, col_339, col_340, col_341, col_342, col_343, col_344, col_345, col_346, col_347, col_348, col_349, col_350, col_351, col_352, col_353, col_354, col_355, col_356, col_357, col_358, col_359, col_360, col_361, col_362, col_363, col_364, col_365, col_366, col_367, col_368, col_369, col_370, col_371, col_372, col_373, col_374, col_375, col_376, col_377, col_378, col_379, col_380, col_381, col_382, col_383, col_384, col_385, col_386, col_387, col_388, col_389, col_390, col_391, col_392, col_393, col_394, col_395, col_396, col_397, col_398, col_399, col_400, col_401, col_402, col_403, col_404, col_405, col_406, col_407, col_408, col_409, col_410, col_411, col_412, col_413, col_414, col_415, col_416, col_417, col_418, col_419, col_420, col_421, col_422, col_423, col_424, col_425, col_426, col_427, col_428, col_429, col_430, col_431, col_432, col_433, col_434, col_435, col_436, col_437, col_438, col_439, col_440, col_441, col_442, col_443, col_444, col_445, col_446, col_447, col_448, col_449, col_450, col_451, col_452, col_453, col_454, col_455, col_456, col_457, col_458, col_459, col_460, col_461, col_462, col_463, col_464, col_465, col_466, col_467, col_468, col_469, col_470, col_471, col_472, col_473, col_474, col_475, col_476, col_477, col_478, col_479, col_480, col_481, col_482, col_483, col_484, col_485, col_486, col_487, col_488, col_489, col_490, col_491, col_492, col_493, col_494, col_495, col_496, col_497, col_498, col_499, col_500, col_501, col_502, col_503, col_504, col_505, col_506, col_507, col_508, col_509, col_510, col_511, col_512, col_513, col_514, col_515, col_516, col_517, col_518, col_519, col_520, col_521, col_522, col_523, col_524, col_525, col_526, col_527, col_528, col_529, col_530, col_531, col_532, col_533, col_534, col_535, col_536, col_537, col_538, col_539, col_540, col_541, col_542, col_543, col_544, col_545, col_546, col_547, col_548, col_549, col_550, col_551, col_552, col_553, col_554, col_555, col_556, col_557, col_558, col_559, col_560, col_561, col_562, col_563, col_564, col_565, col_566, col_567, col_568, col_569, col_570, col_571, col_572, col_573, col_574, col_575, col_576, col_577, col_578, col_579, col_580, col_581, col_582, col_583, col_584, col_585, col_586, col_587, col_588, col_589, col_590, col_591, col_592, col_593, col_594, col_595, col_596, col_597, col_598, col_599, col_600, col_601, col_602, col_603, col_604, col_605, col_606, col_607, col_608, col_609, col_610, col_611, col_612, col_613, col_614, col_615, col_616, col_617, col_618, col_619, col_620, col_621, col_622, col_623, col_624, col_625, col_626, col_627, col_628, col_629, col_630, col_631, col_632, col_633, col_634, col_635, col_636, col_637, col_638, col_639", "save_path": "D:/yuansen/ImPro/impronode/samples/tracking01/tracking08_left_mesh_tracked_data_563x20x1x16.csv", "save_interval": 10, "max_row": 500, "n_cols": 640, "fire_counter": 501, "accumulator_csv": "tracking08.node_87.array_accumulator.csv"}</t>
+          <t>{"col_names": "col_0, col_1, col_2, col_3, col_4, col_5, col_6, col_7, col_8, col_9, col_10, col_11, col_12, col_13, col_14, col_15, col_16, col_17, col_18, col_19, col_20, col_21, col_22, col_23, col_24, col_25, col_26, col_27, col_28, col_29, col_30, col_31, col_32, col_33, col_34, col_35, col_36, col_37, col_38, col_39, col_40, col_41, col_42, col_43, col_44, col_45, col_46, col_47, col_48, col_49, col_50, col_51, col_52, col_53, col_54, col_55, col_56, col_57, col_58, col_59, col_60, col_61, col_62, col_63, col_64, col_65, col_66, col_67, col_68, col_69, col_70, col_71, col_72, col_73, col_74, col_75, col_76, col_77, col_78, col_79, col_80, col_81, col_82, col_83, col_84, col_85, col_86, col_87, col_88, col_89, col_90, col_91, col_92, col_93, col_94, col_95, col_96, col_97, col_98, col_99, col_100, col_101, col_102, col_103, col_104, col_105, col_106, col_107, col_108, col_109, col_110, col_111, col_112, col_113, col_114, col_115, col_116, col_117, col_118, col_119, col_120, col_121, col_122, col_123, col_124, col_125, col_126, col_127, col_128, col_129, col_130, col_131, col_132, col_133, col_134, col_135, col_136, col_137, col_138, col_139, col_140, col_141, col_142, col_143, col_144, col_145, col_146, col_147, col_148, col_149, col_150, col_151, col_152, col_153, col_154, col_155, col_156, col_157, col_158, col_159, col_160, col_161, col_162, col_163, col_164, col_165, col_166, col_167, col_168, col_169, col_170, col_171, col_172, col_173, col_174, col_175, col_176, col_177, col_178, col_179, col_180, col_181, col_182, col_183, col_184, col_185, col_186, col_187, col_188, col_189, col_190, col_191, col_192, col_193, col_194, col_195, col_196, col_197, col_198, col_199, col_200, col_201, col_202, col_203, col_204, col_205, col_206, col_207, col_208, col_209, col_210, col_211, col_212, col_213, col_214, col_215, col_216, col_217, col_218, col_219, col_220, col_221, col_222, col_223, col_224, col_225, col_226, col_227, col_228, col_229, col_230, col_231, col_232, col_233, col_234, col_235, col_236, col_237, col_238, col_239, col_240, col_241, col_242, col_243, col_244, col_245, col_246, col_247, col_248, col_249, col_250, col_251, col_252, col_253, col_254, col_255, col_256, col_257, col_258, col_259, col_260, col_261, col_262, col_263, col_264, col_265, col_266, col_267, col_268, col_269, col_270, col_271, col_272, col_273, col_274, col_275, col_276, col_277, col_278, col_279, col_280, col_281, col_282, col_283, col_284, col_285, col_286, col_287, col_288, col_289, col_290, col_291, col_292, col_293, col_294, col_295, col_296, col_297, col_298, col_299, col_300, col_301, col_302, col_303, col_304, col_305, col_306, col_307, col_308, col_309, col_310, col_311, col_312, col_313, col_314, col_315, col_316, col_317, col_318, col_319, col_320, col_321, col_322, col_323, col_324, col_325, col_326, col_327, col_328, col_329, col_330, col_331, col_332, col_333, col_334, col_335, col_336, col_337, col_338, col_339, col_340, col_341, col_342, col_343, col_344, col_345, col_346, col_347, col_348, col_349, col_350, col_351, col_352, col_353, col_354, col_355, col_356, col_357, col_358, col_359, col_360, col_361, col_362, col_363, col_364, col_365, col_366, col_367, col_368, col_369, col_370, col_371, col_372, col_373, col_374, col_375, col_376, col_377, col_378, col_379, col_380, col_381, col_382, col_383, col_384, col_385, col_386, col_387, col_388, col_389, col_390, col_391, col_392, col_393, col_394, col_395, col_396, col_397, col_398, col_399, col_400, col_401, col_402, col_403, col_404, col_405, col_406, col_407, col_408, col_409, col_410, col_411, col_412, col_413, col_414, col_415, col_416, col_417, col_418, col_419, col_420, col_421, col_422, col_423, col_424, col_425, col_426, col_427, col_428, col_429, col_430, col_431, col_432, col_433, col_434, col_435, col_436, col_437, col_438, col_439, col_440, col_441, col_442, col_443, col_444, col_445, col_446, col_447, col_448, col_449, col_450, col_451, col_452, col_453, col_454, col_455, col_456, col_457, col_458, col_459, col_460, col_461, col_462, col_463, col_464, col_465, col_466, col_467, col_468, col_469, col_470, col_471, col_472, col_473, col_474, col_475, col_476, col_477, col_478, col_479, col_480, col_481, col_482, col_483, col_484, col_485, col_486, col_487, col_488, col_489, col_490, col_491, col_492, col_493, col_494, col_495, col_496, col_497, col_498, col_499, col_500, col_501, col_502, col_503, col_504, col_505, col_506, col_507, col_508, col_509, col_510, col_511, col_512, col_513, col_514, col_515, col_516, col_517, col_518, col_519, col_520, col_521, col_522, col_523, col_524, col_525, col_526, col_527, col_528, col_529, col_530, col_531, col_532, col_533, col_534, col_535, col_536, col_537, col_538, col_539, col_540, col_541, col_542, col_543, col_544, col_545, col_546, col_547, col_548, col_549, col_550, col_551, col_552, col_553, col_554, col_555, col_556, col_557, col_558, col_559, col_560, col_561, col_562, col_563, col_564, col_565, col_566, col_567, col_568, col_569, col_570, col_571, col_572, col_573, col_574, col_575, col_576, col_577, col_578, col_579, col_580, col_581, col_582, col_583, col_584, col_585, col_586, col_587, col_588, col_589, col_590, col_591, col_592, col_593, col_594, col_595, col_596, col_597, col_598, col_599, col_600, col_601, col_602, col_603, col_604, col_605, col_606, col_607, col_608, col_609, col_610, col_611, col_612, col_613, col_614, col_615, col_616, col_617, col_618, col_619, col_620, col_621, col_622, col_623, col_624, col_625, col_626, col_627, col_628, col_629, col_630, col_631, col_632, col_633, col_634, col_635, col_636, col_637, col_638, col_639", "save_path": "D:/yuansen/ImPro/impronode/samples/tracking01/tracking08_left_mesh_tracked_data_563x20x1x16.csv", "save_interval": 10, "max_row": 500, "n_cols": 640, "fire_counter": 507, "accumulator_csv": "tracking08.node_87.array_accumulator.csv"}</t>
         </is>
       </c>
     </row>
@@ -1561,20 +1561,20 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>18</v>
+        <v>187</v>
       </c>
       <c r="E31" t="n">
-        <v>2348</v>
+        <v>2377</v>
       </c>
       <c r="F31" t="n">
-        <v>418</v>
+        <v>529</v>
       </c>
       <c r="G31" t="n">
-        <v>637</v>
+        <v>335</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>{"show_fps": true, "show_coords": true, "show_grid": false, "interpolation": "NEAREST", "marker": "+", "marker_color": [0, 255, 0], "marker_width": 2}</t>
+          <t>{"show_fps": true, "show_coords": true, "show_grid": false, "interpolation": "NEAREST", "marker": "*", "marker_color": [0, 255, 0], "marker_width": 2}</t>
         </is>
       </c>
     </row>
@@ -2071,16 +2071,16 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>792</v>
+        <v>1053</v>
       </c>
       <c r="E46" t="n">
-        <v>2263</v>
+        <v>2391</v>
       </c>
       <c r="F46" t="n">
-        <v>911</v>
+        <v>609</v>
       </c>
       <c r="G46" t="n">
-        <v>725</v>
+        <v>337</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>{"x": "", "y": "", "z": "", "indexing": "ij", "point_size": 1.0, "point_color": "blue", "line_width": 1.0, "line_color": "black", "marker": "o", "line_style": "solid", "show_points": true, "show_lines": true, "show_x_lines": true, "show_y_lines": true, "show_z_lines": true, "preview_enabled": true, "point_sets": [{"enabled": true, "label": "Set 1", "color": "red", "marker": "o", "size": 2.0, "text": "\n\n\n\n\n\n", "grid_lines": true, "grid_dims": "20,1,16", "grid_line_color": "#aa4444", "grid_line_width": 1.0}, {"enabled": true, "label": "Set 2", "color": "blue", "marker": "s", "size": 2.0, "text": "\n\n\n\n\n\n\n", "grid_lines": true, "grid_dims": "20,1,16", "grid_line_color": "blue", "grid_line_width": 1.0}, {"enabled": false, "label": "Set 3", "color": "orange", "marker": "^", "size": 4.0, "text": "\n\n\n\n\n\n\n\n\n\n", "grid_lines": false, "grid_dims": "", "grid_line_color": "#aa8800", "grid_line_width": 1.0}, {"enabled": false, "label": "Set 4", "color": "purple", "marker": "D", "size": 4.0, "text": "\n\n\n\n\n\n\n\n\n\n", "grid_lines": false, "grid_dims": "", "grid_line_color": "#7a4499", "grid_line_width": 1.0}]}</t>
+          <t>{"x": "", "y": "", "z": "", "indexing": "ij", "point_size": 1.0, "point_color": "blue", "line_width": 1.0, "line_color": "black", "marker": "o", "line_style": "solid", "show_points": true, "show_lines": true, "show_x_lines": true, "show_y_lines": true, "show_z_lines": true, "preview_enabled": true, "point_sets": [{"enabled": true, "label": "Set 1", "color": "red", "marker": "o", "size": 2.0, "text": "\n\n\n\n\n\n\n\n", "grid_lines": true, "grid_dims": "20,1,16", "grid_line_color": "#aa4444", "grid_line_width": 1.0}, {"enabled": true, "label": "Set 2", "color": "blue", "marker": "s", "size": 2.0, "text": "\n\n\n\n\n\n\n\n\n", "grid_lines": true, "grid_dims": "20,1,16", "grid_line_color": "blue", "grid_line_width": 1.0}, {"enabled": false, "label": "Set 3", "color": "orange", "marker": "^", "size": 4.0, "text": "\n\n\n\n\n\n\n\n\n\n\n\n", "grid_lines": false, "grid_dims": "", "grid_line_color": "#aa8800", "grid_line_width": 1.0}, {"enabled": false, "label": "Set 4", "color": "purple", "marker": "D", "size": 4.0, "text": "\n\n\n\n\n\n\n\n\n\n\n\n", "grid_lines": false, "grid_dims": "", "grid_line_color": "#7a4499", "grid_line_width": 1.0}]}</t>
         </is>
       </c>
     </row>
@@ -2479,10 +2479,10 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>649</v>
+        <v>115</v>
       </c>
       <c r="E58" t="n">
-        <v>4167</v>
+        <v>4204</v>
       </c>
       <c r="F58" t="n">
         <v>805</v>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>{"x_hint": "1 0 0 ", "normal_hint": "0 1 0 ", "view_mode": "local", "amp_x": 1.0, "amp_y": 1.0, "amp_z": 100.0, "show_points3d": false, "show_lines3d": true, "show_index_labels": true, "surface_field": "exx", "surface_cmap": "jet", "surface_clim_auto": true, "surface_clim_min": -0.01, "surface_clim_max": 0.01, "section_axis": "axis1", "section_index": 4, "section_value": "z", "section_amp": 1.0, "section_xaxis": "index", "field": "vm", "field_res": "gauss", "cmap": "jet_r", "clim_auto": true, "clim_min": 0.0, "clim_max": 1.0, "fps": 10.0, "ts_slots": [{"enabled": true, "source": "Global X", "point_i": 7, "point_j": 5, "mode": "displacement", "color": "red", "marker": "o", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Global X", "point_i": 0, "point_j": 0, "mode": "displacement", "color": "blue", "marker": "s", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "RBM Rotation Y", "point_i": 0, "point_j": 0, "mode": "coord", "color": "green", "marker": "^", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Local Z'", "point_i": 0, "point_j": 0, "mode": "coord", "color": "orange", "marker": "D", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Global X", "point_i": 0, "point_j": 0, "mode": "coord", "color": "purple", "marker": "v", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Global Y", "point_i": 0, "point_j": 0, "mode": "coord", "color": "brown", "marker": "*", "marker_size": 4.0, "line_width": 1.2}], "ts_ylim_auto": false, "ts_ylim_min": -30.0, "ts_ylim_max": 30.0, "img_field": "uz", "img_field_res": "gauss", "img_cmap": "jet", "img_clim_auto": true, "img_clim_min": 0.0, "img_clim_max": 1.0, "img_alpha": 0.45, "video_quality": 95, "video_nstripes": -1}</t>
+          <t>{"x_hint": "1 0 0 ", "normal_hint": "0 1 0 ", "view_mode": "local", "amp_x": 1.0, "amp_y": 1.0, "amp_z": 100.0, "perspective_intensity": 0.35, "show_points3d": false, "show_lines3d": true, "show_index_labels": true, "surface_field": "exx", "surface_cmap": "jet", "surface_clim_auto": true, "surface_clim_min": -0.01, "surface_clim_max": 0.01, "section_axis": "axis1", "section_index": 4, "section_value": "x", "section_amp": 1.0, "section_xaxis": "index", "section_xlabel": "point index along section", "section_ylabel": "local z'", "field": "vm", "field_res": "gauss", "field_shading": "gouraud", "field_xlabel": "local x'", "field_ylabel": "local y'", "cmap": "jet_r", "clim_auto": true, "clim_min": 0.0, "clim_max": 1.0, "fps": 10.0, "ts_slots": [{"enabled": true, "source": "Global X", "point_i": 7, "point_j": 5, "mode": "displacement", "color": "red", "marker": "o", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Global X", "point_i": 0, "point_j": 0, "mode": "displacement", "color": "blue", "marker": "s", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "RBM Rotation Y", "point_i": 0, "point_j": 0, "mode": "coord", "color": "green", "marker": "^", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Local Z'", "point_i": 0, "point_j": 0, "mode": "coord", "color": "orange", "marker": "D", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Global X", "point_i": 0, "point_j": 0, "mode": "coord", "color": "purple", "marker": "v", "marker_size": 4.0, "line_width": 1.2}, {"enabled": false, "source": "Global Y", "point_i": 0, "point_j": 0, "mode": "coord", "color": "brown", "marker": "*", "marker_size": 4.0, "line_width": 1.2}], "ts_ylim_auto": false, "ts_ylim_min": -30.0, "ts_ylim_max": 30.0, "ts_xlabel": "frame index (t)", "ts_ylabel": "value", "img_field": "gxy", "img_field_res": "gauss", "img_shading": "nearest", "img_xlabel": "image x (pixels)", "img_ylabel": "image y (pixels)", "img_cmap": "jet", "img_clim_auto": false, "img_clim_min": -0.015, "img_clim_max": 0.015, "img_alpha": 0.45, "video_quality": 90, "video_nstripes": -1}</t>
         </is>
       </c>
     </row>
@@ -2629,6 +2629,142 @@
       <c r="H62" t="inlineStr">
         <is>
           <t>{"rows_text": ":", "cols_text": ":", "reshape_text": "", "array_viewer_file": "tracking08.node_137.array_viewer.npy"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>node_139</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>array_viewer</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>tm time</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>284</v>
+      </c>
+      <c r="E63" t="n">
+        <v>2226</v>
+      </c>
+      <c r="F63" t="n">
+        <v>101</v>
+      </c>
+      <c r="G63" t="n">
+        <v>80</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>{"rows_text": ":", "cols_text": ":", "reshape_text": "-1", "array_viewer_file": "tracking08.node_139.array_viewer.npy"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>node_141</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>array_accumulator</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>tm time table</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>411</v>
+      </c>
+      <c r="E64" t="n">
+        <v>2222</v>
+      </c>
+      <c r="F64" t="n">
+        <v>164</v>
+      </c>
+      <c r="G64" t="n">
+        <v>80</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>{"col_names": "", "save_path": "", "save_interval": 1, "max_row": 6, "n_cols": 960, "fire_counter": 7, "accumulator_csv": "tracking08.node_141.array_accumulator.csv"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>node_142</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>array_viewer</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>image size</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>97</v>
+      </c>
+      <c r="E65" t="n">
+        <v>492</v>
+      </c>
+      <c r="F65" t="n">
+        <v>108</v>
+      </c>
+      <c r="G65" t="n">
+        <v>80</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>{"rows_text": ":", "cols_text": ":", "reshape_text": "", "array_viewer_file": "tracking08.node_142.array_viewer.npy"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>camera_layout_viewer</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Camera Layout Viewer</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>1122</v>
+      </c>
+      <c r="E66" t="n">
+        <v>294</v>
+      </c>
+      <c r="F66" t="n">
+        <v>220</v>
+      </c>
+      <c r="G66" t="n">
+        <v>270</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>{"grid_xs": "-40:20:400", "grid_ys": "0", "grid_zs": "-40:20:200", "pyr_scale": 1.0, "pyr_width": 1.5, "grid_color": "gray", "grid_width": 1.0, "perspective": 0.0, "show_labels": true, "cam1_color": "#cc2222", "cam2_color": "#2255cc"}</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4670,6 +4806,292 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>node_47</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ctime</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>node_139</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>node_139</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>node_141</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>node_21</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>imgsize</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>node_142</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>array</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>node_21</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>imgsize</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>imgsize1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>node_21</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>cmat</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>cmat1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>node_21</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>dvec</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>dvec1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>node_21</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>rvec</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>rvec1</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>node_21</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>tvec</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>tvec1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>node_24</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>imgsize</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>imgsize2</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>node_24</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>cmat</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>cmat2</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>node_24</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>rvec</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>rvec2</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>node_24</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>dvec</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>dvec2</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>node_24</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>tvec</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>node_143</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>tvec2</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>